<commit_message>
Pipeline run: 2026-07-10 (0 15 * * *)
</commit_message>
<xml_diff>
--- a/workspace/MLB_K_Prop_Model_2026-07-10_am.xlsx
+++ b/workspace/MLB_K_Prop_Model_2026-07-10_am.xlsx
@@ -1796,7 +1796,7 @@
         <v>5.869565217391305</v>
       </c>
       <c r="Q4" s="10" t="n">
-        <v>4.739550511733346</v>
+        <v>4.733324448958688</v>
       </c>
       <c r="R4" s="10" t="n">
         <v>4.25</v>
@@ -1856,7 +1856,7 @@
         <v>4.598253581501229</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>3.761906734494635</v>
+        <v>3.755680671719976</v>
       </c>
       <c r="R5" s="10" t="n">
         <v>4.31</v>
@@ -1916,7 +1916,7 @@
         <v>5.126582526029877</v>
       </c>
       <c r="Q6" s="10" t="n">
-        <v>4.930111964026665</v>
+        <v>4.923885901252007</v>
       </c>
       <c r="R6" s="10" t="n">
         <v>4.62</v>
@@ -1976,7 +1976,7 @@
         <v>3.240000152118397</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>3.166139142662816</v>
+        <v>3.159913079888158</v>
       </c>
       <c r="R7" s="10" t="n">
         <v>3.17</v>
@@ -2036,7 +2036,7 @@
         <v>4.288808900512745</v>
       </c>
       <c r="Q8" s="10" t="n">
-        <v>4.062223613394083</v>
+        <v>4.055997550619425</v>
       </c>
       <c r="R8" s="10" t="n">
         <v>4.62</v>
@@ -2136,7 +2136,7 @@
         <v>5.051613151875805</v>
       </c>
       <c r="Q10" s="21" t="n">
-        <v>4.416759551720121</v>
+        <v>4.410533488945463</v>
       </c>
       <c r="R10" s="21" t="n">
         <v>4.49</v>
@@ -2196,7 +2196,7 @@
         <v>3.375000221975933</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>3.895847414336508</v>
+        <v>3.88962135156185</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>4.34</v>
@@ -2256,7 +2256,7 @@
         <v>4.281553398058253</v>
       </c>
       <c r="Q12" s="10" t="n">
-        <v>4.673383352594469</v>
+        <v>4.66715728981981</v>
       </c>
       <c r="R12" s="10" t="n">
         <v>3.67</v>
@@ -2356,7 +2356,7 @@
         <v>4.790322893802156</v>
       </c>
       <c r="Q14" s="10" t="n">
-        <v>3.833695018418625</v>
+        <v>3.827468955643967</v>
       </c>
       <c r="R14" s="10" t="n">
         <v>4.56</v>
@@ -2416,7 +2416,7 @@
         <v>2.61</v>
       </c>
       <c r="Q15" s="10" t="n">
-        <v>3.829985294342041</v>
+        <v>3.823759231567383</v>
       </c>
       <c r="R15" s="10" t="n">
         <v>4.68</v>
@@ -2476,7 +2476,7 @@
         <v>2.801886994119824</v>
       </c>
       <c r="Q16" s="10" t="n">
-        <v>3.101117368455713</v>
+        <v>3.094891305681054</v>
       </c>
       <c r="R16" s="10" t="n">
         <v>3.22</v>
@@ -2536,7 +2536,7 @@
         <v>4.002695500102812</v>
       </c>
       <c r="Q17" s="10" t="n">
-        <v>3.863920619613675</v>
+        <v>3.857694556839017</v>
       </c>
       <c r="R17" s="10" t="n">
         <v>3.78</v>
@@ -2596,7 +2596,7 @@
         <v>2.609665501524787</v>
       </c>
       <c r="Q18" s="10" t="n">
-        <v>3.610691627962086</v>
+        <v>3.604465565187428</v>
       </c>
       <c r="R18" s="10" t="n">
         <v>3.7</v>
@@ -2656,7 +2656,7 @@
         <v>3.730263345129281</v>
       </c>
       <c r="Q19" s="10" t="n">
-        <v>3.524590577808445</v>
+        <v>3.518364515033787</v>
       </c>
       <c r="R19" s="10" t="n">
         <v>3.41</v>
@@ -2716,7 +2716,7 @@
         <v>7.04347834431285</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>6.119985329882699</v>
+        <v>6.113759267108041</v>
       </c>
       <c r="R20" s="10" t="n">
         <v>4.05</v>
@@ -2776,7 +2776,7 @@
         <v>3.55743252412519</v>
       </c>
       <c r="Q21" s="10" t="n">
-        <v>3.738228553520493</v>
+        <v>3.732002490745835</v>
       </c>
       <c r="R21" s="10" t="n">
         <v>3.72</v>
@@ -2836,7 +2836,7 @@
         <v>3.375000146302316</v>
       </c>
       <c r="Q22" s="21" t="n">
-        <v>4.449530806521741</v>
+        <v>4.443304743747083</v>
       </c>
       <c r="R22" s="21" t="n">
         <v>3.41</v>
@@ -2896,7 +2896,7 @@
         <v>3.347107701822368</v>
       </c>
       <c r="Q23" s="21" t="n">
-        <v>4.657175498141943</v>
+        <v>4.650949435367285</v>
       </c>
       <c r="R23" s="21" t="n">
         <v>4.87</v>
@@ -2956,7 +2956,7 @@
         <v>8.064935864033474</v>
       </c>
       <c r="Q24" s="21" t="n">
-        <v>5.145959521055764</v>
+        <v>5.139733458281106</v>
       </c>
       <c r="R24" s="21" t="n">
         <v>7.22</v>
@@ -3016,7 +3016,7 @@
         <v>4.426229508196721</v>
       </c>
       <c r="Q25" s="10" t="n">
-        <v>5.103591851719091</v>
+        <v>5.097365788944432</v>
       </c>
       <c r="R25" s="10" t="n">
         <v>4.46</v>
@@ -3076,7 +3076,7 @@
         <v>2.273684210526316</v>
       </c>
       <c r="Q26" s="10" t="n">
-        <v>2.898932662763094</v>
+        <v>2.892706599988436</v>
       </c>
       <c r="R26" s="10" t="n">
         <v>3.44</v>
@@ -3136,7 +3136,7 @@
         <v>3.857143084383524</v>
       </c>
       <c r="Q27" s="10" t="n">
-        <v>4.1045413369024</v>
+        <v>4.098315274127741</v>
       </c>
       <c r="R27" s="10" t="n">
         <v>5.56</v>
@@ -3276,7 +3276,7 @@
         <v>2.25</v>
       </c>
       <c r="Q30" s="10" t="n">
-        <v>4.00887418323093</v>
+        <v>4.002648120456271</v>
       </c>
       <c r="R30" s="10" t="n">
         <v>5.01</v>
@@ -3336,7 +3336,7 @@
         <v>1.785992270918442</v>
       </c>
       <c r="Q31" s="10" t="n">
-        <v>2.629712906246783</v>
+        <v>2.623486843472124</v>
       </c>
       <c r="R31" s="10" t="n">
         <v>2.7</v>
@@ -3390,13 +3390,13 @@
         <v>24.8</v>
       </c>
       <c r="O32" s="21" t="n">
-        <v>45.9</v>
+        <v>46</v>
       </c>
       <c r="P32" s="21" t="n">
         <v>6.948529606665712</v>
       </c>
       <c r="Q32" s="21" t="n">
-        <v>5.039102995230667</v>
+        <v>5.032876932456008</v>
       </c>
       <c r="R32" s="21" t="n">
         <v>4.87</v>
@@ -3456,7 +3456,7 @@
         <v>3.452459199911044</v>
       </c>
       <c r="Q33" s="10" t="n">
-        <v>4.703591935896679</v>
+        <v>4.69736587312202</v>
       </c>
       <c r="R33" s="10" t="n">
         <v>4.56</v>
@@ -4825,33 +4825,33 @@
         <v>5.5</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>-101</v>
+        <v>105</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>-127</v>
+        <v>-134</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="H5" s="28" t="n">
-        <v>-102</v>
+        <v>100</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>-125</v>
+        <v>-128</v>
       </c>
       <c r="J5" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="K5" s="9" t="n">
-        <v>-125</v>
+      <c r="K5" s="29" t="n">
+        <v>-134</v>
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M5" s="9" t="n">
-        <v>-125</v>
+        <v>-128</v>
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
@@ -4923,10 +4923,10 @@
         <v>5.5</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>-152</v>
+        <v>-146</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>5.5</v>
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c r="M7" s="9" t="n">
-        <v>-152</v>
+        <v>-146</v>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
@@ -4972,10 +4972,10 @@
         <v>6.5</v>
       </c>
       <c r="E8" s="28" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>-141</v>
+        <v>-145</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>6.5</v>
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="M8" s="9" t="n">
-        <v>-141</v>
+        <v>-145</v>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
@@ -5021,10 +5021,10 @@
         <v>5.5</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>-152</v>
+        <v>-144</v>
       </c>
       <c r="G9" s="28" t="n">
         <v>5.5</v>
@@ -5047,7 +5047,7 @@
         </is>
       </c>
       <c r="M9" s="9" t="n">
-        <v>-152</v>
+        <v>-144</v>
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
@@ -5093,37 +5093,37 @@
         <v>4.5</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>-139</v>
+        <v>-160</v>
       </c>
       <c r="G11" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="H11" s="28" t="n">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>-148</v>
+        <v>-158</v>
       </c>
       <c r="J11" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="K11" s="29" t="n">
-        <v>-148</v>
+        <v>-160</v>
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>-158</v>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
           <t>FD</t>
-        </is>
-      </c>
-      <c r="M11" s="9" t="n">
-        <v>-139</v>
-      </c>
-      <c r="N11" s="9" t="inlineStr">
-        <is>
-          <t>DK</t>
         </is>
       </c>
     </row>
@@ -5142,37 +5142,37 @@
         <v>4.5</v>
       </c>
       <c r="E12" s="28" t="n">
-        <v>-101</v>
+        <v>107</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>-126</v>
+        <v>-136</v>
       </c>
       <c r="G12" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="H12" s="28" t="n">
-        <v>-104</v>
+        <v>106</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>-122</v>
+        <v>-136</v>
       </c>
       <c r="J12" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="K12" s="9" t="n">
-        <v>-122</v>
+      <c r="K12" s="29" t="n">
+        <v>-136</v>
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M12" s="9" t="n">
-        <v>-122</v>
+        <v>-136</v>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
     </row>
@@ -5191,10 +5191,10 @@
         <v>5.5</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>-109</v>
+        <v>-118</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>-117</v>
+        <v>-108</v>
       </c>
       <c r="G13" s="28" t="n">
         <v>5.5</v>
@@ -5209,19 +5209,19 @@
         <v>5.5</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M13" s="9" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
     </row>
@@ -5240,10 +5240,10 @@
         <v>6.5</v>
       </c>
       <c r="E14" s="28" t="n">
-        <v>-110</v>
+        <v>-107</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>-115</v>
+        <v>-119</v>
       </c>
       <c r="G14" s="28" t="n">
         <v>6.5</v>
@@ -5258,7 +5258,7 @@
         <v>6.5</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>-115</v>
+        <v>-119</v>
       </c>
       <c r="L14" s="9" t="inlineStr">
         <is>
@@ -5266,7 +5266,7 @@
         </is>
       </c>
       <c r="M14" s="9" t="n">
-        <v>-115</v>
+        <v>-119</v>
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
@@ -5289,10 +5289,10 @@
         <v>4.5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>-110</v>
+        <v>-104</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>-116</v>
+        <v>-123</v>
       </c>
       <c r="G15" s="28" t="n">
         <v>4.5</v>
@@ -5307,7 +5307,7 @@
         <v>4.5</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>-116</v>
+        <v>-123</v>
       </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
@@ -5315,7 +5315,7 @@
         </is>
       </c>
       <c r="M15" s="9" t="n">
-        <v>-116</v>
+        <v>-123</v>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
@@ -5338,25 +5338,25 @@
         <v>4.5</v>
       </c>
       <c r="E16" s="28" t="n">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>-140</v>
+        <v>-157</v>
       </c>
       <c r="G16" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="H16" s="28" t="n">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>-146</v>
+        <v>-160</v>
       </c>
       <c r="J16" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="K16" s="29" t="n">
-        <v>-146</v>
+        <v>-160</v>
       </c>
       <c r="L16" s="9" t="inlineStr">
         <is>
@@ -5364,7 +5364,7 @@
         </is>
       </c>
       <c r="M16" s="9" t="n">
-        <v>-140</v>
+        <v>-157</v>
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
@@ -5387,33 +5387,33 @@
         <v>5.5</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>-106</v>
+        <v>104</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>-121</v>
+        <v>-132</v>
       </c>
       <c r="G17" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="H17" s="28" t="n">
-        <v>-113</v>
+        <v>-102</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>-113</v>
+        <v>-125</v>
       </c>
       <c r="J17" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="K17" s="9" t="n">
-        <v>-113</v>
+      <c r="K17" s="29" t="n">
+        <v>-132</v>
       </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M17" s="9" t="n">
-        <v>-113</v>
+        <v>-125</v>
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
@@ -5436,25 +5436,25 @@
         <v>5.5</v>
       </c>
       <c r="E18" s="28" t="n">
-        <v>-113</v>
+        <v>118</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>-113</v>
+        <v>-150</v>
       </c>
       <c r="G18" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="H18" s="28" t="n">
-        <v>-104</v>
+        <v>110</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>-122</v>
+        <v>-140</v>
       </c>
       <c r="J18" s="28" t="n">
         <v>5.5</v>
       </c>
-      <c r="K18" s="9" t="n">
-        <v>-113</v>
+      <c r="K18" s="29" t="n">
+        <v>-150</v>
       </c>
       <c r="L18" s="9" t="inlineStr">
         <is>
@@ -5462,11 +5462,11 @@
         </is>
       </c>
       <c r="M18" s="9" t="n">
-        <v>-113</v>
+        <v>-140</v>
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
         <v>-135</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G19" s="28" t="n">
         <v>5.5</v>
@@ -5503,7 +5503,7 @@
         <v>5.5</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L19" s="9" t="inlineStr">
         <is>
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="M19" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
@@ -5534,37 +5534,37 @@
         <v>6.5</v>
       </c>
       <c r="E20" s="28" t="n">
-        <v>-121</v>
+        <v>-123</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="G20" s="28" t="n">
         <v>6.5</v>
       </c>
       <c r="H20" s="28" t="n">
-        <v>-130</v>
+        <v>-115</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>102</v>
+        <v>-111</v>
       </c>
       <c r="J20" s="28" t="n">
         <v>6.5</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>102</v>
+        <v>-104</v>
       </c>
       <c r="L20" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M20" s="9" t="n">
-        <v>102</v>
+        <v>-104</v>
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
     </row>
@@ -5606,37 +5606,37 @@
         <v>5.5</v>
       </c>
       <c r="E22" s="28" t="n">
-        <v>-152</v>
+        <v>-145</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="G22" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="H22" s="28" t="n">
-        <v>-142</v>
+        <v>-150</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="J22" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FD</t>
         </is>
       </c>
       <c r="M22" s="9" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -5655,10 +5655,10 @@
         <v>5.5</v>
       </c>
       <c r="E23" s="28" t="n">
-        <v>-156</v>
+        <v>-133</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="G23" s="28" t="n">
         <v>5.5</v>
@@ -5673,7 +5673,7 @@
         <v>5.5</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="M23" s="9" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
@@ -5704,10 +5704,10 @@
         <v>3.5</v>
       </c>
       <c r="E24" s="28" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>-176</v>
+        <v>-171</v>
       </c>
       <c r="G24" s="28" t="n">
         <v>3.5</v>
@@ -5722,19 +5722,19 @@
         <v>3.5</v>
       </c>
       <c r="K24" s="29" t="n">
-        <v>-176</v>
+        <v>-174</v>
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
+          <t>FD</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="n">
+        <v>-171</v>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
           <t>DK</t>
-        </is>
-      </c>
-      <c r="M24" s="9" t="n">
-        <v>-174</v>
-      </c>
-      <c r="N24" s="9" t="inlineStr">
-        <is>
-          <t>FD</t>
         </is>
       </c>
     </row>
@@ -5753,33 +5753,33 @@
         <v>4.5</v>
       </c>
       <c r="E25" s="28" t="n">
-        <v>-105</v>
+        <v>131</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>-122</v>
+        <v>-168</v>
       </c>
       <c r="G25" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="H25" s="28" t="n">
-        <v>-130</v>
+        <v>124</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>102</v>
+        <v>-160</v>
       </c>
       <c r="J25" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="K25" s="9" t="n">
-        <v>102</v>
+      <c r="K25" s="29" t="n">
+        <v>-168</v>
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M25" s="9" t="n">
-        <v>102</v>
+        <v>-160</v>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
@@ -5802,33 +5802,33 @@
         <v>5.5</v>
       </c>
       <c r="E26" s="28" t="n">
-        <v>-105</v>
+        <v>102</v>
       </c>
       <c r="F26" s="12" t="n">
-        <v>-122</v>
+        <v>-130</v>
       </c>
       <c r="G26" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="H26" s="28" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>-130</v>
+        <v>-132</v>
       </c>
       <c r="J26" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="K26" s="29" t="n">
+        <v>-132</v>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>FD</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="n">
         <v>-130</v>
-      </c>
-      <c r="L26" s="9" t="inlineStr">
-        <is>
-          <t>FD</t>
-        </is>
-      </c>
-      <c r="M26" s="9" t="n">
-        <v>-122</v>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
@@ -5851,25 +5851,25 @@
         <v>6.5</v>
       </c>
       <c r="E27" s="28" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F27" s="12" t="n">
-        <v>-163</v>
+        <v>-153</v>
       </c>
       <c r="G27" s="28" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="H27" s="28" t="n">
-        <v>-164</v>
+        <v>118</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>128</v>
+        <v>-150</v>
       </c>
       <c r="J27" s="28" t="n">
         <v>6.5</v>
       </c>
       <c r="K27" s="29" t="n">
-        <v>-163</v>
+        <v>-153</v>
       </c>
       <c r="L27" s="9" t="inlineStr">
         <is>
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="M27" s="9" t="n">
-        <v>128</v>
+        <v>-150</v>
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
@@ -5900,37 +5900,37 @@
         <v>3.5</v>
       </c>
       <c r="E28" s="28" t="n">
-        <v>-158</v>
+        <v>-155</v>
       </c>
       <c r="F28" s="12" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G28" s="28" t="n">
         <v>3.5</v>
       </c>
       <c r="H28" s="28" t="n">
-        <v>-146</v>
+        <v>-156</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="J28" s="28" t="n">
         <v>3.5</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L28" s="9" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FD</t>
         </is>
       </c>
       <c r="M28" s="9" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N28" s="9" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -5949,33 +5949,33 @@
         <v>4.5</v>
       </c>
       <c r="E29" s="28" t="n">
-        <v>-106</v>
+        <v>107</v>
       </c>
       <c r="F29" s="12" t="n">
-        <v>-121</v>
+        <v>-137</v>
       </c>
       <c r="G29" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="H29" s="28" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>-128</v>
+        <v>-148</v>
       </c>
       <c r="J29" s="28" t="n">
         <v>4.5</v>
       </c>
-      <c r="K29" s="9" t="n">
-        <v>-121</v>
+      <c r="K29" s="29" t="n">
+        <v>-148</v>
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FD</t>
         </is>
       </c>
       <c r="M29" s="9" t="n">
-        <v>-121</v>
+        <v>-137</v>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
@@ -5998,25 +5998,25 @@
         <v>3.5</v>
       </c>
       <c r="E30" s="28" t="n">
-        <v>-138</v>
+        <v>-141</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G30" s="28" t="n">
         <v>3.5</v>
       </c>
       <c r="H30" s="28" t="n">
-        <v>-120</v>
+        <v>-128</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>-106</v>
+        <v>100</v>
       </c>
       <c r="J30" s="28" t="n">
         <v>3.5</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
@@ -6024,7 +6024,7 @@
         </is>
       </c>
       <c r="M30" s="9" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
@@ -6047,25 +6047,25 @@
         <v>4.5</v>
       </c>
       <c r="E31" s="28" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>-156</v>
+        <v>-163</v>
       </c>
       <c r="G31" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="H31" s="28" t="n">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>-148</v>
+        <v>-162</v>
       </c>
       <c r="J31" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="K31" s="29" t="n">
-        <v>-156</v>
+        <v>-163</v>
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
@@ -6073,7 +6073,7 @@
         </is>
       </c>
       <c r="M31" s="9" t="n">
-        <v>-148</v>
+        <v>-162</v>
       </c>
       <c r="N31" s="9" t="inlineStr">
         <is>
@@ -6096,37 +6096,37 @@
         <v>6.5</v>
       </c>
       <c r="E32" s="28" t="n">
-        <v>-104</v>
+        <v>121</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>-123</v>
+        <v>-155</v>
       </c>
       <c r="G32" s="28" t="n">
         <v>6.5</v>
       </c>
       <c r="H32" s="28" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>-150</v>
+        <v>-148</v>
       </c>
       <c r="J32" s="28" t="n">
         <v>6.5</v>
       </c>
       <c r="K32" s="29" t="n">
-        <v>-150</v>
+        <v>-155</v>
       </c>
       <c r="L32" s="9" t="inlineStr">
         <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="M32" s="9" t="n">
+        <v>-148</v>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
           <t>FD</t>
-        </is>
-      </c>
-      <c r="M32" s="9" t="n">
-        <v>-123</v>
-      </c>
-      <c r="N32" s="9" t="inlineStr">
-        <is>
-          <t>DK</t>
         </is>
       </c>
     </row>
@@ -6145,25 +6145,25 @@
         <v>4.5</v>
       </c>
       <c r="E33" s="28" t="n">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>-164</v>
+        <v>-161</v>
       </c>
       <c r="G33" s="28" t="n">
         <v>3.5</v>
       </c>
       <c r="H33" s="28" t="n">
-        <v>-148</v>
+        <v>-170</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="J33" s="28" t="n">
         <v>4.5</v>
       </c>
       <c r="K33" s="29" t="n">
-        <v>-164</v>
+        <v>-161</v>
       </c>
       <c r="L33" s="9" t="inlineStr">
         <is>
@@ -6171,7 +6171,7 @@
         </is>
       </c>
       <c r="M33" s="9" t="n">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="N33" s="9" t="inlineStr">
         <is>
@@ -6194,37 +6194,37 @@
         <v>5.5</v>
       </c>
       <c r="E34" s="28" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>-125</v>
+        <v>-124</v>
       </c>
       <c r="G34" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="H34" s="28" t="n">
-        <v>-111</v>
+        <v>100</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>-115</v>
+        <v>-128</v>
       </c>
       <c r="J34" s="28" t="n">
         <v>5.5</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>-115</v>
+        <v>-124</v>
       </c>
       <c r="L34" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="M34" s="9" t="n">
-        <v>-115</v>
+        <v>-124</v>
       </c>
       <c r="N34" s="9" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>DK</t>
         </is>
       </c>
     </row>
@@ -6355,7 +6355,7 @@
         </is>
       </c>
       <c r="J5" s="30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -6394,7 +6394,7 @@
         </is>
       </c>
       <c r="J6" s="30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -6433,7 +6433,7 @@
         </is>
       </c>
       <c r="J7" s="30" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -6472,7 +6472,7 @@
         </is>
       </c>
       <c r="J8" s="30" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="J9" s="30" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="J10" s="30" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -6589,7 +6589,7 @@
         </is>
       </c>
       <c r="J11" s="30" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -6628,7 +6628,7 @@
         </is>
       </c>
       <c r="J12" s="30" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -6667,7 +6667,7 @@
         </is>
       </c>
       <c r="J13" s="30" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
@@ -6706,7 +6706,7 @@
         </is>
       </c>
       <c r="J14" s="30" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -6901,7 +6901,7 @@
         </is>
       </c>
       <c r="J19" s="30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -6940,7 +6940,7 @@
         </is>
       </c>
       <c r="J20" s="30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -7213,7 +7213,7 @@
         </is>
       </c>
       <c r="J27" s="30" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28">
@@ -7252,7 +7252,7 @@
         </is>
       </c>
       <c r="J28" s="30" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>-141 (DK)</t>
+          <t>-145 (DK)</t>
         </is>
       </c>
       <c r="I5" s="35" t="n">
@@ -9414,7 +9414,7 @@
         <v>-0.63</v>
       </c>
       <c r="M5" s="37" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="N5" s="14" t="inlineStr">
         <is>
@@ -9453,12 +9453,12 @@
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>-163 (DK)</t>
+          <t>-153 (DK)</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>128 (FD)</t>
+          <t>-150 (FD)</t>
         </is>
       </c>
       <c r="I6" s="35" t="n">
@@ -9474,7 +9474,7 @@
         <v>-0.58</v>
       </c>
       <c r="M6" s="37" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="N6" s="14" t="inlineStr">
         <is>
@@ -9483,7 +9483,7 @@
       </c>
       <c r="O6" s="33" t="inlineStr">
         <is>
-          <t>Gate PASS: residual -1.13 ≤ -0.75, qualifying Under -163 (DK), Rule 5 pass, PPD ≤ 50%</t>
+          <t>Gate PASS: residual -1.13 ≤ -0.75, qualifying Under -153 (DK), Rule 5 pass, PPD ≤ 50%</t>
         </is>
       </c>
     </row>
@@ -9513,12 +9513,12 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>-150 (FD)</t>
+          <t>-155 (DK)</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>-123 (DK)</t>
+          <t>-148 (FD)</t>
         </is>
       </c>
       <c r="I7" s="35" t="n">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="O7" s="33" t="inlineStr">
         <is>
-          <t>Gate PASS: residual -1.06 ≤ -0.75, qualifying Under -150 (FD), Rule 5 pass, PPD ≤ 50%</t>
+          <t>Gate PASS: residual -1.06 ≤ -0.75, qualifying Under -155 (DK), Rule 5 pass, PPD ≤ 50%</t>
         </is>
       </c>
     </row>

</xml_diff>